<commit_message>
Vorsorgeaufwand: Fix broken selection + EP01/EP02 logic + QoL
- Replace dropdown ✓ with free text "x" input (was unusable - 3 clicks)
- Fix SUMPRODUCT formulas: check <>'' instead of ='✓'
- EP01/EP02 priority: EP02 supersedes EP01 in results
- Add TEXTJOIN summary of selected G-numbers in result header
- Add reset hint (select row 2, press Del)
- Update note text for EP01/EP02

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/Vorsorgeaufwand_2026.xlsx
+++ b/Vorsorgeaufwand_2026.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,7 +48,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00B71C1C"/>
-      <sz val="9"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -80,8 +80,21 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F3460"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="0028A745"/>
       <sz val="9"/>
     </font>
     <font>
@@ -187,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -199,7 +212,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom" textRotation="90" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -210,8 +223,8 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -236,19 +249,22 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -264,7 +280,7 @@
         <name val="Calibri"/>
         <b val="1"/>
         <color rgb="00B71C1C"/>
-        <sz val="9"/>
+        <sz val="11"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -636,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AS33"/>
+  <dimension ref="A1:AS34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -698,10 +714,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="25" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>▼ G-Untersuchung auswählen (✓)</t>
+          <t>▼ "x" eingeben zum Auswählen →</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
@@ -747,7 +763,7 @@
       <c r="AP2" s="4" t="n"/>
       <c r="AQ2" s="4" t="n"/>
       <c r="AR2" s="5">
-        <f>IF(COUNTA(AS4:AS31)&gt;0,"✓ "&amp;COUNTA(AS4:AS31)&amp;" Untersuchung(en) erforderlich","Bitte G-Nummern in Zeile 3 auswählen (✓)")</f>
+        <f>IF(COUNTA(AS4:AS31)&gt;0,"✓ "&amp;COUNTA(AS4:AS31)&amp;" Untersuchung(en) erforderlich","← x eingeben bei den gewünschten G-Nummern")</f>
         <v/>
       </c>
     </row>
@@ -967,10 +983,9 @@
           <t>FEV1</t>
         </is>
       </c>
-      <c r="AS3" s="8" t="inlineStr">
-        <is>
-          <t>Untersuchung</t>
-        </is>
+      <c r="AS3" s="8">
+        <f>IF(COUNTA(B2:AQ2)&gt;0,"Gewählt: "&amp;TEXTJOIN(", ",TRUE,IF(B2:AQ2&lt;&gt;"",B3:AQ3,"")),"← Untersuchungen")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
@@ -1183,7 +1198,7 @@
       </c>
       <c r="AR4" s="11" t="n"/>
       <c r="AS4" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B4:AQ4&lt;&gt;""))&gt;0,A4,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B4:AQ4&lt;&gt;""))&gt;0,A4,"")</f>
         <v/>
       </c>
     </row>
@@ -1401,7 +1416,7 @@
       </c>
       <c r="AR5" s="15" t="n"/>
       <c r="AS5" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B5:AQ5&lt;&gt;""))&gt;0,A5,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B5:AQ5&lt;&gt;""))&gt;0,A5,"")</f>
         <v/>
       </c>
     </row>
@@ -1479,7 +1494,7 @@
       </c>
       <c r="AR6" s="11" t="n"/>
       <c r="AS6" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B6:AQ6&lt;&gt;""))&gt;0,A6,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B6:AQ6&lt;&gt;""))&gt;0,A6,"")</f>
         <v/>
       </c>
     </row>
@@ -1541,7 +1556,7 @@
       <c r="AQ7" s="14" t="n"/>
       <c r="AR7" s="15" t="n"/>
       <c r="AS7" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B7:AQ7&lt;&gt;""))&gt;0,A7,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B7:AQ7&lt;&gt;""))&gt;0,A7,"")</f>
         <v/>
       </c>
     </row>
@@ -1599,7 +1614,7 @@
       <c r="AQ8" s="10" t="n"/>
       <c r="AR8" s="11" t="n"/>
       <c r="AS8" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B8:AQ8&lt;&gt;""))&gt;0,A8,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B8:AQ8&lt;&gt;""))&gt;0,A8,"")</f>
         <v/>
       </c>
     </row>
@@ -1801,7 +1816,7 @@
       </c>
       <c r="AR9" s="15" t="n"/>
       <c r="AS9" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B9:AQ9&lt;&gt;""))&gt;0,A9,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B9:AQ9&lt;&gt;""))&gt;0,A9,"")</f>
         <v/>
       </c>
     </row>
@@ -1867,7 +1882,7 @@
       <c r="AQ10" s="10" t="n"/>
       <c r="AR10" s="11" t="n"/>
       <c r="AS10" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B10:AQ10&lt;&gt;""))&gt;0,A10,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B10:AQ10&lt;&gt;""))&gt;0,A10,"")</f>
         <v/>
       </c>
     </row>
@@ -1925,7 +1940,7 @@
       <c r="AQ11" s="14" t="n"/>
       <c r="AR11" s="15" t="n"/>
       <c r="AS11" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B11:AQ11&lt;&gt;""))&gt;0,A11,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B11:AQ11&lt;&gt;""))&gt;0,A11,"")</f>
         <v/>
       </c>
     </row>
@@ -2075,7 +2090,7 @@
       </c>
       <c r="AR12" s="11" t="n"/>
       <c r="AS12" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B12:AQ12&lt;&gt;""))&gt;0,A12,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B12:AQ12&lt;&gt;""))&gt;0,A12,"")</f>
         <v/>
       </c>
     </row>
@@ -2169,7 +2184,7 @@
       </c>
       <c r="AR13" s="15" t="n"/>
       <c r="AS13" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B13:AQ13&lt;&gt;""))&gt;0,A13,"")</f>
+        <f>IF(AND(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B13:AQ13&lt;&gt;""))&gt;0,SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B14:AQ14&lt;&gt;""))=0),A13,"")</f>
         <v/>
       </c>
     </row>
@@ -2263,7 +2278,7 @@
       <c r="AQ14" s="10" t="n"/>
       <c r="AR14" s="11" t="n"/>
       <c r="AS14" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B14:AQ14&lt;&gt;""))&gt;0,A14,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B14:AQ14&lt;&gt;""))&gt;0,A14&amp;" (ersetzt EP01)","")</f>
         <v/>
       </c>
     </row>
@@ -2369,7 +2384,7 @@
       </c>
       <c r="AR15" s="15" t="n"/>
       <c r="AS15" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B15:AQ15&lt;&gt;""))&gt;0,A15,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B15:AQ15&lt;&gt;""))&gt;0,A15,"")</f>
         <v/>
       </c>
     </row>
@@ -2435,7 +2450,7 @@
       </c>
       <c r="AR16" s="11" t="n"/>
       <c r="AS16" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B16:AQ16&lt;&gt;""))&gt;0,A16,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B16:AQ16&lt;&gt;""))&gt;0,A16,"")</f>
         <v/>
       </c>
     </row>
@@ -2553,7 +2568,7 @@
       <c r="AQ17" s="14" t="n"/>
       <c r="AR17" s="15" t="n"/>
       <c r="AS17" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B17:AQ17&lt;&gt;""))&gt;0,A17,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B17:AQ17&lt;&gt;""))&gt;0,A17,"")</f>
         <v/>
       </c>
     </row>
@@ -2651,7 +2666,7 @@
       <c r="AQ18" s="10" t="n"/>
       <c r="AR18" s="11" t="n"/>
       <c r="AS18" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B18:AQ18&lt;&gt;""))&gt;0,A18,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B18:AQ18&lt;&gt;""))&gt;0,A18,"")</f>
         <v/>
       </c>
     </row>
@@ -2737,7 +2752,7 @@
       <c r="AQ19" s="14" t="n"/>
       <c r="AR19" s="15" t="n"/>
       <c r="AS19" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B19:AQ19&lt;&gt;""))&gt;0,A19,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B19:AQ19&lt;&gt;""))&gt;0,A19,"")</f>
         <v/>
       </c>
     </row>
@@ -2795,7 +2810,7 @@
       <c r="AQ20" s="10" t="n"/>
       <c r="AR20" s="11" t="n"/>
       <c r="AS20" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B20:AQ20&lt;&gt;""))&gt;0,A20,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B20:AQ20&lt;&gt;""))&gt;0,A20,"")</f>
         <v/>
       </c>
     </row>
@@ -2997,7 +3012,7 @@
       </c>
       <c r="AR21" s="15" t="n"/>
       <c r="AS21" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B21:AQ21&lt;&gt;""))&gt;0,A21,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B21:AQ21&lt;&gt;""))&gt;0,A21,"")</f>
         <v/>
       </c>
     </row>
@@ -3087,7 +3102,7 @@
       <c r="AQ22" s="10" t="n"/>
       <c r="AR22" s="11" t="n"/>
       <c r="AS22" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B22:AQ22&lt;&gt;""))&gt;0,A22,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B22:AQ22&lt;&gt;""))&gt;0,A22,"")</f>
         <v/>
       </c>
     </row>
@@ -3157,7 +3172,7 @@
       <c r="AQ23" s="14" t="n"/>
       <c r="AR23" s="15" t="n"/>
       <c r="AS23" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B23:AQ23&lt;&gt;""))&gt;0,A23,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B23:AQ23&lt;&gt;""))&gt;0,A23,"")</f>
         <v/>
       </c>
     </row>
@@ -3219,7 +3234,7 @@
       <c r="AQ24" s="10" t="n"/>
       <c r="AR24" s="11" t="n"/>
       <c r="AS24" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B24:AQ24&lt;&gt;""))&gt;0,A24,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B24:AQ24&lt;&gt;""))&gt;0,A24,"")</f>
         <v/>
       </c>
     </row>
@@ -3289,7 +3304,7 @@
       <c r="AQ25" s="14" t="n"/>
       <c r="AR25" s="15" t="n"/>
       <c r="AS25" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B25:AQ25&lt;&gt;""))&gt;0,A25,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B25:AQ25&lt;&gt;""))&gt;0,A25,"")</f>
         <v/>
       </c>
     </row>
@@ -3347,7 +3362,7 @@
       <c r="AQ26" s="10" t="n"/>
       <c r="AR26" s="11" t="n"/>
       <c r="AS26" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B26:AQ26&lt;&gt;""))&gt;0,A26,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B26:AQ26&lt;&gt;""))&gt;0,A26,"")</f>
         <v/>
       </c>
     </row>
@@ -3413,7 +3428,7 @@
       <c r="AQ27" s="14" t="n"/>
       <c r="AR27" s="15" t="n"/>
       <c r="AS27" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B27:AQ27&lt;&gt;""))&gt;0,A27,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B27:AQ27&lt;&gt;""))&gt;0,A27,"")</f>
         <v/>
       </c>
     </row>
@@ -3635,7 +3650,7 @@
       </c>
       <c r="AR28" s="11" t="n"/>
       <c r="AS28" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B28:AQ28&lt;&gt;""))&gt;0,A28,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B28:AQ28&lt;&gt;""))&gt;0,A28,"")</f>
         <v/>
       </c>
     </row>
@@ -3857,7 +3872,7 @@
       </c>
       <c r="AR29" s="15" t="n"/>
       <c r="AS29" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B29:AQ29&lt;&gt;""))&gt;0,A29,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B29:AQ29&lt;&gt;""))&gt;0,A29,"")</f>
         <v/>
       </c>
     </row>
@@ -3951,7 +3966,7 @@
       <c r="AQ30" s="10" t="n"/>
       <c r="AR30" s="11" t="n"/>
       <c r="AS30" s="12">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B30:AQ30&lt;&gt;""))&gt;0,A30,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B30:AQ30&lt;&gt;""))&gt;0,A30,"")</f>
         <v/>
       </c>
     </row>
@@ -4045,34 +4060,37 @@
       <c r="AQ31" s="14" t="n"/>
       <c r="AR31" s="15" t="n"/>
       <c r="AS31" s="16">
-        <f>IF(SUMPRODUCT(($B$2:$AQ$2="✓")*(B31:AQ31&lt;&gt;""))&gt;0,A31,"")</f>
+        <f>IF(SUMPRODUCT(($B$2:$AQ$2&lt;&gt;"")*(B31:AQ31&lt;&gt;""))&gt;0,A31,"")</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>Hinweis: Gelbe Zellen = EP01 (Labor Blut). Wenn EP02 erforderlich, ersetzt EP02 den EP01. Belastungs-EKG bei G35-Varianten nur ab 45 Jahre ("45J.").</t>
+          <t>Hinweis: Gelbe Zellen = EP01/EP02 (Labor Blut). Wenn EP02 erforderlich, ersetzt EP02 den EP01. Belastungs-EKG bei G35-Varianten nur ab 45 Jahre ("45J.").</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Zurücksetzen: Markieren Sie Zeile 2 (grüne Auswahlzeile), drücken Sie Entf um alle Auswahlen zu löschen.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A34:AQ34"/>
+    <mergeCell ref="AR2:AS2"/>
+    <mergeCell ref="AR1:AS1"/>
+    <mergeCell ref="A33:AQ33"/>
     <mergeCell ref="A1:AQ1"/>
-    <mergeCell ref="AR1:AS1"/>
-    <mergeCell ref="AR2:AS2"/>
-    <mergeCell ref="A33:AQ33"/>
   </mergeCells>
   <conditionalFormatting sqref="B2:AQ2">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0" stopIfTrue="0">
-      <formula>"✓"</formula>
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>B2&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:AQ2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="G-Untersuchung" prompt="✓ = auswählen" type="list">
-      <formula1>"✓"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -4104,34 +4122,34 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>G-Nr.</t>
         </is>
       </c>
-      <c r="B1" s="19" t="inlineStr">
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>Bereich</t>
         </is>
       </c>
-      <c r="C1" s="19" t="inlineStr">
+      <c r="C1" s="20" t="inlineStr">
         <is>
           <t>Substanz</t>
         </is>
       </c>
-      <c r="D1" s="19" t="inlineStr">
+      <c r="D1" s="20" t="inlineStr">
         <is>
           <t>Probenmaterial</t>
         </is>
       </c>
-      <c r="E1" s="19" t="inlineStr">
+      <c r="E1" s="20" t="inlineStr">
         <is>
           <t>Bedingungen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>G7</t>
         </is>
@@ -4146,7 +4164,7 @@
           <t>COHb</t>
         </is>
       </c>
-      <c r="D2" s="21" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>Fingersensor</t>
         </is>
@@ -4154,7 +4172,7 @@
       <c r="E2" s="12" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>G8</t>
         </is>
@@ -4169,11 +4187,11 @@
           <t>Benzol</t>
         </is>
       </c>
-      <c r="D3" s="23" t="inlineStr"/>
+      <c r="D3" s="24" t="inlineStr"/>
       <c r="E3" s="16" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>G27</t>
         </is>
@@ -4188,11 +4206,11 @@
           <t>kein Wert hinterlegt</t>
         </is>
       </c>
-      <c r="D4" s="21" t="inlineStr"/>
+      <c r="D4" s="22" t="inlineStr"/>
       <c r="E4" s="12" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>G29</t>
         </is>
@@ -4207,11 +4225,11 @@
           <t>kein Wert hinterlegt</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr"/>
+      <c r="D5" s="24" t="inlineStr"/>
       <c r="E5" s="16" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr"/>
+      <c r="A6" s="21" t="inlineStr"/>
       <c r="B6" s="12" t="inlineStr">
         <is>
           <t>QM</t>
@@ -4222,11 +4240,11 @@
           <t>kein Wert hinterlegt</t>
         </is>
       </c>
-      <c r="D6" s="21" t="inlineStr"/>
+      <c r="D6" s="22" t="inlineStr"/>
       <c r="E6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>G38</t>
         </is>
@@ -4241,11 +4259,11 @@
           <t>Nickel im Urin</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr"/>
+      <c r="D7" s="24" t="inlineStr"/>
       <c r="E7" s="16" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>G45</t>
         </is>
@@ -4256,7 +4274,7 @@
           <t>Styrol</t>
         </is>
       </c>
-      <c r="D8" s="21" t="inlineStr"/>
+      <c r="D8" s="22" t="inlineStr"/>
       <c r="E8" s="12" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix checkmark positions in Vorsorgeaufwand to match 2023 original
7 checkmarks were incorrect compared to the 2023 source file:
- Labor Blut EP01: add missing G21
- Ruhe EKG: replace incorrect G7 with G21
- Röntgen: remove incorrect G40
- Rhinoskopie: add missing G38
- ODIN-Bogen: remove incorrect G27 and G42

https://claude.ai/code/session_016bQ6N1upLzi6x6LMsZZWnq
</commit_message>
<xml_diff>
--- a/Vorsorgeaufwand_2026.xlsx
+++ b/Vorsorgeaufwand_2026.xlsx
@@ -2112,7 +2112,11 @@
       <c r="G13" s="14" t="n"/>
       <c r="H13" s="14" t="n"/>
       <c r="I13" s="14" t="n"/>
-      <c r="J13" s="14" t="n"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="n"/>
       <c r="L13" s="14" t="n"/>
       <c r="M13" s="14" t="n"/>
@@ -2581,16 +2585,16 @@
       <c r="B18" s="10" t="n"/>
       <c r="C18" s="10" t="n"/>
       <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="E18" s="10" t="n"/>
       <c r="F18" s="10" t="n"/>
       <c r="G18" s="10" t="n"/>
       <c r="H18" s="10" t="n"/>
       <c r="I18" s="10" t="n"/>
-      <c r="J18" s="10" t="n"/>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K18" s="10" t="n"/>
       <c r="L18" s="10" t="n"/>
       <c r="M18" s="10" t="n"/>
@@ -3077,11 +3081,7 @@
       <c r="Z22" s="10" t="n"/>
       <c r="AA22" s="10" t="n"/>
       <c r="AB22" s="10" t="n"/>
-      <c r="AC22" s="10" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="AC22" s="10" t="n"/>
       <c r="AD22" s="10" t="n"/>
       <c r="AE22" s="10" t="n"/>
       <c r="AF22" s="10" t="n"/>
@@ -3343,7 +3343,11 @@
       <c r="X26" s="10" t="n"/>
       <c r="Y26" s="10" t="n"/>
       <c r="Z26" s="10" t="n"/>
-      <c r="AA26" s="10" t="n"/>
+      <c r="AA26" s="10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="AB26" s="10" t="n"/>
       <c r="AC26" s="10" t="n"/>
       <c r="AD26" s="10" t="n"/>
@@ -3914,11 +3918,7 @@
       <c r="O30" s="10" t="n"/>
       <c r="P30" s="10" t="n"/>
       <c r="Q30" s="10" t="n"/>
-      <c r="R30" s="10" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="R30" s="10" t="n"/>
       <c r="S30" s="10" t="n"/>
       <c r="T30" s="10" t="n"/>
       <c r="U30" s="10" t="inlineStr">
@@ -3943,11 +3943,7 @@
         </is>
       </c>
       <c r="AD30" s="10" t="n"/>
-      <c r="AE30" s="10" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="AE30" s="10" t="n"/>
       <c r="AF30" s="10" t="inlineStr">
         <is>
           <t>x</t>

</xml_diff>